<commit_message>
better background and model comparison results
</commit_message>
<xml_diff>
--- a/Modelling/Paper_experiments/models_ml_per_writer.xlsx
+++ b/Modelling/Paper_experiments/models_ml_per_writer.xlsx
@@ -398,22 +398,22 @@
         </is>
       </c>
       <c r="B2">
-        <v>-2364.923331974381</v>
+        <v>-946.7077080527584</v>
       </c>
       <c r="C2">
-        <v>-2364.324183724846</v>
+        <v>-941.5706004928683</v>
       </c>
       <c r="D2">
-        <v>-2328.505459191701</v>
+        <v>-903.7087308943978</v>
       </c>
       <c r="E2">
-        <v>-2236.86470373102</v>
+        <v>-903.1922128012383</v>
       </c>
       <c r="F2">
-        <v>-2242.633934210578</v>
+        <v>-908.0784719053572</v>
       </c>
       <c r="G2">
-        <v>-2212.637904159773</v>
+        <v>-878.3887434916976</v>
       </c>
     </row>
     <row r="3">
@@ -423,22 +423,22 @@
         </is>
       </c>
       <c r="B3">
-        <v>-1430.757623191424</v>
+        <v>-1147.721940528187</v>
       </c>
       <c r="C3">
-        <v>-1427.571815676498</v>
+        <v>-1141.329307633127</v>
       </c>
       <c r="D3">
-        <v>-1379.570243013302</v>
+        <v>-1095.092450817289</v>
       </c>
       <c r="E3">
-        <v>-1381.815931579549</v>
+        <v>-1085.184004228589</v>
       </c>
       <c r="F3">
-        <v>-1376.064918648797</v>
+        <v>-1070.527808968715</v>
       </c>
       <c r="G3">
-        <v>-1331.818132414804</v>
+        <v>-1028.984432021305</v>
       </c>
     </row>
     <row r="4">
@@ -448,22 +448,22 @@
         </is>
       </c>
       <c r="B4">
-        <v>-1056.7859401157</v>
+        <v>-948.023690411808</v>
       </c>
       <c r="C4">
-        <v>-1055.514252299259</v>
+        <v>-944.267393912099</v>
       </c>
       <c r="D4">
-        <v>-1028.335660620144</v>
+        <v>-916.9060143371822</v>
       </c>
       <c r="E4">
-        <v>-1027.294977140183</v>
+        <v>-894.8898789663489</v>
       </c>
       <c r="F4">
-        <v>-1032.66574402102</v>
+        <v>-889.9143581126777</v>
       </c>
       <c r="G4">
-        <v>-1008.871490345787</v>
+        <v>-868.7918720328275</v>
       </c>
     </row>
     <row r="5">
@@ -473,22 +473,22 @@
         </is>
       </c>
       <c r="B5">
-        <v>-1075.616418985163</v>
+        <v>-1025.420401805119</v>
       </c>
       <c r="C5">
-        <v>-1074.51380411387</v>
+        <v>-1018.662996575121</v>
       </c>
       <c r="D5">
-        <v>-1048.737963967538</v>
+        <v>-979.1243372504788</v>
       </c>
       <c r="E5">
-        <v>-1048.956149173148</v>
+        <v>-989.6074035448518</v>
       </c>
       <c r="F5">
-        <v>-1055.139148770053</v>
+        <v>-977.4302149967168</v>
       </c>
       <c r="G5">
-        <v>-1033.802574076855</v>
+        <v>-942.1824812576552</v>
       </c>
     </row>
     <row r="6">
@@ -498,22 +498,22 @@
         </is>
       </c>
       <c r="B6">
-        <v>-1188.767313508051</v>
+        <v>-696.2743976224605</v>
       </c>
       <c r="C6">
-        <v>-1185.81197565757</v>
+        <v>-690.5313968594147</v>
       </c>
       <c r="D6">
-        <v>-1142.692452635398</v>
+        <v>-675.5636559622769</v>
       </c>
       <c r="E6">
-        <v>-1180.369457322771</v>
+        <v>-676.2558691192415</v>
       </c>
       <c r="F6">
-        <v>-1176.700616980153</v>
+        <v>-664.2261897350287</v>
       </c>
       <c r="G6">
-        <v>-1136.112906495296</v>
+        <v>-652.122721033909</v>
       </c>
     </row>
     <row r="7">
@@ -523,22 +523,22 @@
         </is>
       </c>
       <c r="B7">
-        <v>-981.1031225428183</v>
+        <v>-893.8171037362446</v>
       </c>
       <c r="C7">
-        <v>-980.337109942154</v>
+        <v>-887.3393471941916</v>
       </c>
       <c r="D7">
-        <v>-948.4472209357435</v>
+        <v>-857.3512228955194</v>
       </c>
       <c r="E7">
-        <v>-966.1705076676768</v>
+        <v>-875.1481820938878</v>
       </c>
       <c r="F7">
-        <v>-969.3323564598213</v>
+        <v>-864.4916686006181</v>
       </c>
       <c r="G7">
-        <v>-941.4712758138726</v>
+        <v>-838.5056005653502</v>
       </c>
     </row>
     <row r="8">
@@ -548,22 +548,22 @@
         </is>
       </c>
       <c r="B8">
-        <v>-1020.588037752388</v>
+        <v>-768.2998215371242</v>
       </c>
       <c r="C8">
-        <v>-1017.314687192955</v>
+        <v>-759.3278435578192</v>
       </c>
       <c r="D8">
-        <v>-988.8364351943438</v>
+        <v>-737.7006460793883</v>
       </c>
       <c r="E8">
-        <v>-958.55164442905</v>
+        <v>-688.6639180618457</v>
       </c>
       <c r="F8">
-        <v>-958.8585168698647</v>
+        <v>-677.0134931491824</v>
       </c>
       <c r="G8">
-        <v>-934.7914105779802</v>
+        <v>-662.6139332886593</v>
       </c>
     </row>
     <row r="9">
@@ -573,22 +573,22 @@
         </is>
       </c>
       <c r="B9">
-        <v>-1040.280053194671</v>
+        <v>-922.5495143225157</v>
       </c>
       <c r="C9">
-        <v>-1039.162173464953</v>
+        <v>-922.6259950449087</v>
       </c>
       <c r="D9">
-        <v>-1003.718449102953</v>
+        <v>-887.189018777811</v>
       </c>
       <c r="E9">
-        <v>-984.5403731866376</v>
+        <v>-835.3645871864927</v>
       </c>
       <c r="F9">
-        <v>-983.6214458130199</v>
+        <v>-825.7015886357487</v>
       </c>
       <c r="G9">
-        <v>-951.6039071380434</v>
+        <v>-796.8412538405101</v>
       </c>
     </row>
     <row r="10">
@@ -598,22 +598,22 @@
         </is>
       </c>
       <c r="B10">
-        <v>-1183.620674367118</v>
+        <v>-930.4006529878005</v>
       </c>
       <c r="C10">
-        <v>-1181.634860389932</v>
+        <v>-927.5349276204402</v>
       </c>
       <c r="D10">
-        <v>-1146.530084654959</v>
+        <v>-896.833872832772</v>
       </c>
       <c r="E10">
-        <v>-1108.862243611508</v>
+        <v>-881.188129460328</v>
       </c>
       <c r="F10">
-        <v>-1112.606362609401</v>
+        <v>-869.0633065536082</v>
       </c>
       <c r="G10">
-        <v>-1082.514426669265</v>
+        <v>-841.7839303557955</v>
       </c>
     </row>
     <row r="11">
@@ -623,22 +623,22 @@
         </is>
       </c>
       <c r="B11">
-        <v>-1145.780907733244</v>
+        <v>-962.4983445708706</v>
       </c>
       <c r="C11">
-        <v>-1143.274628208918</v>
+        <v>-956.7370890505181</v>
       </c>
       <c r="D11">
-        <v>-1106.703765055611</v>
+        <v>-925.2074123793657</v>
       </c>
       <c r="E11">
-        <v>-1100.198429699661</v>
+        <v>-903.4645953679636</v>
       </c>
       <c r="F11">
-        <v>-1097.977458039893</v>
+        <v>-892.7060819839912</v>
       </c>
       <c r="G11">
-        <v>-1063.486931738003</v>
+        <v>-866.9679849282207</v>
       </c>
     </row>
     <row r="12">
@@ -648,22 +648,22 @@
         </is>
       </c>
       <c r="B12">
-        <v>-1093.69032926624</v>
+        <v>-1046.208477887839</v>
       </c>
       <c r="C12">
-        <v>-1091.771959434177</v>
+        <v>-1040.460026855854</v>
       </c>
       <c r="D12">
-        <v>-1054.287117442299</v>
+        <v>-991.7082236329965</v>
       </c>
       <c r="E12">
-        <v>-1078.624950771137</v>
+        <v>-1035.894840064841</v>
       </c>
       <c r="F12">
-        <v>-1076.520965001687</v>
+        <v>-1024.412221702297</v>
       </c>
       <c r="G12">
-        <v>-1039.498643029037</v>
+        <v>-977.5339012759011</v>
       </c>
     </row>
     <row r="13">
@@ -673,22 +673,22 @@
         </is>
       </c>
       <c r="B13">
-        <v>-1103.152039281104</v>
+        <v>-1131.086672591406</v>
       </c>
       <c r="C13">
-        <v>-1098.425726830566</v>
+        <v>-1121.53808410245</v>
       </c>
       <c r="D13">
-        <v>-1057.728669038562</v>
+        <v>-1066.988332786406</v>
       </c>
       <c r="E13">
-        <v>-1127.630267275052</v>
+        <v>-1130.002913541694</v>
       </c>
       <c r="F13">
-        <v>-1118.010016800833</v>
+        <v>-1104.111646193815</v>
       </c>
       <c r="G13">
-        <v>-1078.920878170742</v>
+        <v>-1051.139354435989</v>
       </c>
     </row>
     <row r="14">
@@ -698,22 +698,22 @@
         </is>
       </c>
       <c r="B14">
-        <v>-1288.379779980795</v>
+        <v>-697.2093112369575</v>
       </c>
       <c r="C14">
-        <v>-1287.891949195184</v>
+        <v>-693.5723700007967</v>
       </c>
       <c r="D14">
-        <v>-1262.836303532709</v>
+        <v>-692.239336987752</v>
       </c>
       <c r="E14">
-        <v>-1168.676330495281</v>
+        <v>-620.5613276019084</v>
       </c>
       <c r="F14">
-        <v>-1167.568727676305</v>
+        <v>-604.3896757214175</v>
       </c>
       <c r="G14">
-        <v>-1152.053055201519</v>
+        <v>-612.09478471847</v>
       </c>
     </row>
     <row r="15">
@@ -723,22 +723,22 @@
         </is>
       </c>
       <c r="B15">
-        <v>-1109.083874246022</v>
+        <v>-790.5870822391861</v>
       </c>
       <c r="C15">
-        <v>-1107.530822066613</v>
+        <v>-787.006269272177</v>
       </c>
       <c r="D15">
-        <v>-1076.859226184444</v>
+        <v>-775.8968321600223</v>
       </c>
       <c r="E15">
-        <v>-980.9249264899853</v>
+        <v>-682.3522012225452</v>
       </c>
       <c r="F15">
-        <v>-982.8233248442461</v>
+        <v>-683.9350461853438</v>
       </c>
       <c r="G15">
-        <v>-959.4870164199735</v>
+        <v>-679.499072758526</v>
       </c>
     </row>
     <row r="16">
@@ -748,72 +748,72 @@
         </is>
       </c>
       <c r="B16">
-        <v>-1002.143178051697</v>
+        <v>-822.5546460293006</v>
       </c>
       <c r="C16">
-        <v>-993.9917528685343</v>
+        <v>-809.2927378642858</v>
       </c>
       <c r="D16">
-        <v>-960.2133327467151</v>
+        <v>-773.384119939112</v>
       </c>
       <c r="E16">
-        <v>-971.7085667339251</v>
+        <v>-788.0032544682816</v>
       </c>
       <c r="F16">
-        <v>-958.4137294823186</v>
+        <v>-763.0208669263366</v>
       </c>
       <c r="G16">
-        <v>-926.8493947001599</v>
+        <v>-732.0731840633796</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>87</t>
         </is>
       </c>
       <c r="B17">
-        <v>-956.4040308448798</v>
+        <v>-729.8476925787619</v>
       </c>
       <c r="C17">
-        <v>-955.6715902097075</v>
+        <v>-718.6580292303943</v>
       </c>
       <c r="D17">
-        <v>-932.9926703950572</v>
+        <v>-704.2692221577983</v>
       </c>
       <c r="E17">
-        <v>-894.9821161994167</v>
+        <v>-696.6983646712468</v>
       </c>
       <c r="F17">
-        <v>-899.4084911819579</v>
+        <v>-682.8202283995394</v>
       </c>
       <c r="G17">
-        <v>-882.4786027095465</v>
+        <v>-675.4870564921221</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>88</t>
         </is>
       </c>
       <c r="B18">
-        <v>-928.7215768276438</v>
+        <v>-924.8925328978746</v>
       </c>
       <c r="C18">
-        <v>-921.509915521822</v>
+        <v>-922.5478298243905</v>
       </c>
       <c r="D18">
-        <v>-899.2979490728014</v>
+        <v>-903.234622460961</v>
       </c>
       <c r="E18">
-        <v>-917.4063476858022</v>
+        <v>-877.0553726556076</v>
       </c>
       <c r="F18">
-        <v>-904.1306239624192</v>
+        <v>-867.6329238439724</v>
       </c>
       <c r="G18">
-        <v>-887.7470505274334</v>
+        <v>-853.8139958003018</v>
       </c>
     </row>
     <row r="19">
@@ -823,22 +823,22 @@
         </is>
       </c>
       <c r="B19">
-        <v>-888.2145285247677</v>
+        <v>-778.7769326031448</v>
       </c>
       <c r="C19">
-        <v>-887.6412264349744</v>
+        <v>-773.6342369665939</v>
       </c>
       <c r="D19">
-        <v>-866.367496900275</v>
+        <v>-763.83985060219</v>
       </c>
       <c r="E19">
-        <v>-800.1137180397444</v>
+        <v>-671.4281945145693</v>
       </c>
       <c r="F19">
-        <v>-808.2129451067196</v>
+        <v>-663.1445902614503</v>
       </c>
       <c r="G19">
-        <v>-796.6491651348789</v>
+        <v>-663.5668346196619</v>
       </c>
     </row>
     <row r="20">
@@ -848,22 +848,22 @@
         </is>
       </c>
       <c r="B20">
-        <v>-992.8518977258659</v>
+        <v>-762.8690190990371</v>
       </c>
       <c r="C20">
-        <v>-991.4442521397493</v>
+        <v>-757.8484371236162</v>
       </c>
       <c r="D20">
-        <v>-963.1095856285613</v>
+        <v>-749.8655132282291</v>
       </c>
       <c r="E20">
-        <v>-921.1262968434461</v>
+        <v>-698.0867552809485</v>
       </c>
       <c r="F20">
-        <v>-923.2628522921879</v>
+        <v>-692.4506024680948</v>
       </c>
       <c r="G20">
-        <v>-901.1196765981765</v>
+        <v>-692.3380635288651</v>
       </c>
     </row>
     <row r="21">
@@ -873,22 +873,22 @@
         </is>
       </c>
       <c r="B21">
-        <v>-986.2706786617003</v>
+        <v>-852.8391789207043</v>
       </c>
       <c r="C21">
-        <v>-984.6298899402909</v>
+        <v>-846.5678772437351</v>
       </c>
       <c r="D21">
-        <v>-945.2987234421381</v>
+        <v>-822.2996318557099</v>
       </c>
       <c r="E21">
-        <v>-964.7150151847849</v>
+        <v>-826.6954903280879</v>
       </c>
       <c r="F21">
-        <v>-964.2447719070557</v>
+        <v>-813.4883369067677</v>
       </c>
       <c r="G21">
-        <v>-929.3326351593257</v>
+        <v>-793.1233863707755</v>
       </c>
     </row>
     <row r="22">
@@ -898,22 +898,22 @@
         </is>
       </c>
       <c r="B22">
-        <v>-1089.952333435966</v>
+        <v>-852.5968190458362</v>
       </c>
       <c r="C22">
-        <v>-1087.099891080671</v>
+        <v>-843.5270523281956</v>
       </c>
       <c r="D22">
-        <v>-1042.290264345975</v>
+        <v>-815.6790932857832</v>
       </c>
       <c r="E22">
-        <v>-1109.838363454717</v>
+        <v>-852.9209467216259</v>
       </c>
       <c r="F22">
-        <v>-1105.168998983635</v>
+        <v>-826.8160642101354</v>
       </c>
       <c r="G22">
-        <v>-1062.577661147841</v>
+        <v>-803.1888804535205</v>
       </c>
     </row>
     <row r="23">
@@ -923,22 +923,22 @@
         </is>
       </c>
       <c r="B23">
-        <v>-1350.224996451423</v>
+        <v>-1064.27328023294</v>
       </c>
       <c r="C23">
-        <v>-1347.493955839517</v>
+        <v>-1059.659663119743</v>
       </c>
       <c r="D23">
-        <v>-1308.331018892127</v>
+        <v>-1025.097788170717</v>
       </c>
       <c r="E23">
-        <v>-1278.181417648866</v>
+        <v>-983.6768746484539</v>
       </c>
       <c r="F23">
-        <v>-1274.19514886132</v>
+        <v>-978.7818108836987</v>
       </c>
       <c r="G23">
-        <v>-1236.292800067561</v>
+        <v>-949.192539993341</v>
       </c>
     </row>
     <row r="24">
@@ -948,22 +948,22 @@
         </is>
       </c>
       <c r="B24">
-        <v>-1178.575432864829</v>
+        <v>-869.7801198092868</v>
       </c>
       <c r="C24">
-        <v>-1176.105368336479</v>
+        <v>-862.7271105374325</v>
       </c>
       <c r="D24">
-        <v>-1131.494728778227</v>
+        <v>-832.2454592260032</v>
       </c>
       <c r="E24">
-        <v>-1149.820696015061</v>
+        <v>-856.928953186596</v>
       </c>
       <c r="F24">
-        <v>-1146.93709041719</v>
+        <v>-844.3855103806869</v>
       </c>
       <c r="G24">
-        <v>-1107.647386357212</v>
+        <v>-817.5065714434297</v>
       </c>
     </row>
     <row r="25">
@@ -973,22 +973,22 @@
         </is>
       </c>
       <c r="B25">
-        <v>-891.2912961967741</v>
+        <v>-699.4436672178408</v>
       </c>
       <c r="C25">
-        <v>-888.0008741316378</v>
+        <v>-695.2186908954628</v>
       </c>
       <c r="D25">
-        <v>-848.6963091972584</v>
+        <v>-659.9383346646312</v>
       </c>
       <c r="E25">
-        <v>-910.4452545738474</v>
+        <v>-717.701928430712</v>
       </c>
       <c r="F25">
-        <v>-903.9604864054933</v>
+        <v>-694.3829983432004</v>
       </c>
       <c r="G25">
-        <v>-867.9846733068828</v>
+        <v>-660.84353498256</v>
       </c>
     </row>
     <row r="26">
@@ -998,22 +998,22 @@
         </is>
       </c>
       <c r="B26">
-        <v>-1162.047127369641</v>
+        <v>-782.3639525421853</v>
       </c>
       <c r="C26">
-        <v>-1161.250490007714</v>
+        <v>-777.7328004541843</v>
       </c>
       <c r="D26">
-        <v>-1132.604205823162</v>
+        <v>-759.6033903084775</v>
       </c>
       <c r="E26">
-        <v>-1116.268733217471</v>
+        <v>-755.3833165483719</v>
       </c>
       <c r="F26">
-        <v>-1119.941771029222</v>
+        <v>-745.5464728020071</v>
       </c>
       <c r="G26">
-        <v>-1098.419064555418</v>
+        <v>-730.4015458589719</v>
       </c>
     </row>
     <row r="27">
@@ -1023,22 +1023,22 @@
         </is>
       </c>
       <c r="B27">
-        <v>-1169.281663616988</v>
+        <v>-950.5269348961466</v>
       </c>
       <c r="C27">
-        <v>-1167.002198284022</v>
+        <v>-944.5872397742932</v>
       </c>
       <c r="D27">
-        <v>-1127.498244912468</v>
+        <v>-907.5176090592155</v>
       </c>
       <c r="E27">
-        <v>-1062.282856855312</v>
+        <v>-883.7857040202106</v>
       </c>
       <c r="F27">
-        <v>-1063.845496534479</v>
+        <v>-873.4827845907112</v>
       </c>
       <c r="G27">
-        <v>-1033.37476405386</v>
+        <v>-838.8690515240924</v>
       </c>
     </row>
     <row r="28">
@@ -1048,22 +1048,22 @@
         </is>
       </c>
       <c r="B28">
-        <v>-1016.369387133889</v>
+        <v>-808.3993611569729</v>
       </c>
       <c r="C28">
-        <v>-1015.787978224754</v>
+        <v>-805.4857455826715</v>
       </c>
       <c r="D28">
-        <v>-986.8856565892745</v>
+        <v>-784.8249744806735</v>
       </c>
       <c r="E28">
-        <v>-943.4319646452149</v>
+        <v>-721.9789262553126</v>
       </c>
       <c r="F28">
-        <v>-949.6069120436647</v>
+        <v>-729.1119044455952</v>
       </c>
       <c r="G28">
-        <v>-929.5223421112387</v>
+        <v>-717.8470362920785</v>
       </c>
     </row>
     <row r="29">
@@ -1073,22 +1073,22 @@
         </is>
       </c>
       <c r="B29">
-        <v>-1070.720358497527</v>
+        <v>-1133.652769743994</v>
       </c>
       <c r="C29">
-        <v>-1067.919420766291</v>
+        <v>-1124.518355522148</v>
       </c>
       <c r="D29">
-        <v>-1022.067357014573</v>
+        <v>-1076.932636995445</v>
       </c>
       <c r="E29">
-        <v>-1090.180291964617</v>
+        <v>-1122.238425179743</v>
       </c>
       <c r="F29">
-        <v>-1084.385249270346</v>
+        <v>-1105.607748455585</v>
       </c>
       <c r="G29">
-        <v>-1040.527492862936</v>
+        <v>-1059.450666211216</v>
       </c>
     </row>
     <row r="30">
@@ -1098,22 +1098,22 @@
         </is>
       </c>
       <c r="B30">
-        <v>-1104.926470672652</v>
+        <v>-891.201405143419</v>
       </c>
       <c r="C30">
-        <v>-1102.725911009691</v>
+        <v>-885.5236189286851</v>
       </c>
       <c r="D30">
-        <v>-1065.403864093031</v>
+        <v>-852.5745045864866</v>
       </c>
       <c r="E30">
-        <v>-1100.611812273552</v>
+        <v>-886.1216925036891</v>
       </c>
       <c r="F30">
-        <v>-1098.922100627881</v>
+        <v>-868.5893718434858</v>
       </c>
       <c r="G30">
-        <v>-1065.998368523856</v>
+        <v>-840.1924208335031</v>
       </c>
     </row>
     <row r="31">
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="B31">
-        <v>-1054.301100925114</v>
+        <v>-985.0640338066833</v>
       </c>
       <c r="C31">
-        <v>-1052.109555388487</v>
+        <v>-979.2988990331046</v>
       </c>
       <c r="D31">
-        <v>-1013.270470274536</v>
+        <v>-938.5791957896913</v>
       </c>
       <c r="E31">
-        <v>-981.7079222068722</v>
+        <v>-919.0064309709668</v>
       </c>
       <c r="F31">
-        <v>-982.5589416892667</v>
+        <v>-912.0567390647091</v>
       </c>
       <c r="G31">
-        <v>-947.1392465154356</v>
+        <v>-877.6594973214889</v>
       </c>
     </row>
     <row r="32">
@@ -1148,22 +1148,22 @@
         </is>
       </c>
       <c r="B32">
-        <v>-1197.676703127887</v>
+        <v>-838.7710747461612</v>
       </c>
       <c r="C32">
-        <v>-1195.565888239244</v>
+        <v>-835.2890953690176</v>
       </c>
       <c r="D32">
-        <v>-1154.292637700815</v>
+        <v>-803.9269170486904</v>
       </c>
       <c r="E32">
-        <v>-1162.857338506447</v>
+        <v>-784.7650775617761</v>
       </c>
       <c r="F32">
-        <v>-1161.07066667082</v>
+        <v>-779.4841892208817</v>
       </c>
       <c r="G32">
-        <v>-1126.885376235056</v>
+        <v>-758.7329916210638</v>
       </c>
     </row>
     <row r="33">
@@ -1173,22 +1173,22 @@
         </is>
       </c>
       <c r="B33">
-        <v>-1122.526025871465</v>
+        <v>-998.6585646581244</v>
       </c>
       <c r="C33">
-        <v>-1117.257855843149</v>
+        <v>-990.3766126834072</v>
       </c>
       <c r="D33">
-        <v>-1084.553479151992</v>
+        <v>-951.6727874001066</v>
       </c>
       <c r="E33">
-        <v>-1137.867012953099</v>
+        <v>-991.0027620689401</v>
       </c>
       <c r="F33">
-        <v>-1128.810538237171</v>
+        <v>-1019.21075304506</v>
       </c>
       <c r="G33">
-        <v>-1097.830453320606</v>
+        <v>-977.5975606812488</v>
       </c>
     </row>
     <row r="34">
@@ -1198,22 +1198,22 @@
         </is>
       </c>
       <c r="B34">
-        <v>-1001.334117717249</v>
+        <v>-718.2286795555735</v>
       </c>
       <c r="C34">
-        <v>-1000.823531769009</v>
+        <v>-712.5879716814674</v>
       </c>
       <c r="D34">
-        <v>-975.8056469584733</v>
+        <v>-706.9415688415809</v>
       </c>
       <c r="E34">
-        <v>-962.2616095946245</v>
+        <v>-675.6580514206206</v>
       </c>
       <c r="F34">
-        <v>-967.6403190740502</v>
+        <v>-662.825183350637</v>
       </c>
       <c r="G34">
-        <v>-949.0862907527518</v>
+        <v>-665.3234529066547</v>
       </c>
     </row>
     <row r="35">
@@ -1223,22 +1223,22 @@
         </is>
       </c>
       <c r="B35">
-        <v>-1243.717829149085</v>
+        <v>-1100.790026098261</v>
       </c>
       <c r="C35">
-        <v>-1241.902327261755</v>
+        <v>-1116.60790628376</v>
       </c>
       <c r="D35">
-        <v>-1213.084030786434</v>
+        <v>-1088.590675326239</v>
       </c>
       <c r="E35">
-        <v>-1040.777093634546</v>
+        <v>-950.3713741371292</v>
       </c>
       <c r="F35">
-        <v>-1044.464717287956</v>
+        <v>-1016.130145029408</v>
       </c>
       <c r="G35">
-        <v>-1017.808178958188</v>
+        <v>-989.6683531039262</v>
       </c>
     </row>
     <row r="36">
@@ -1248,22 +1248,22 @@
         </is>
       </c>
       <c r="B36">
-        <v>-1307.173538606986</v>
+        <v>-1162.043201541487</v>
       </c>
       <c r="C36">
-        <v>-1304.18648800105</v>
+        <v>-1155.549660777723</v>
       </c>
       <c r="D36">
-        <v>-1260.299021032132</v>
+        <v>-1114.113128166513</v>
       </c>
       <c r="E36">
-        <v>-1306.119174204401</v>
+        <v>-1114.532957733752</v>
       </c>
       <c r="F36">
-        <v>-1297.128966840007</v>
+        <v>-1103.215350518983</v>
       </c>
       <c r="G36">
-        <v>-1253.346412202053</v>
+        <v>-1065.196560614777</v>
       </c>
     </row>
     <row r="37">
@@ -1273,22 +1273,22 @@
         </is>
       </c>
       <c r="B37">
-        <v>-1397.902477974942</v>
+        <v>-1197.942948314892</v>
       </c>
       <c r="C37">
-        <v>-1395.067735111376</v>
+        <v>-1192.712791226716</v>
       </c>
       <c r="D37">
-        <v>-1340.791990209631</v>
+        <v>-1136.936039102449</v>
       </c>
       <c r="E37">
-        <v>-1239.980926165003</v>
+        <v>-1047.636447607001</v>
       </c>
       <c r="F37">
-        <v>-1238.003310779409</v>
+        <v>-1059.708609031092</v>
       </c>
       <c r="G37">
-        <v>-1192.447408487711</v>
+        <v>-1007.446542962861</v>
       </c>
     </row>
     <row r="38">
@@ -1298,22 +1298,22 @@
         </is>
       </c>
       <c r="B38">
-        <v>-878.5290042837897</v>
+        <v>-816.7023136309913</v>
       </c>
       <c r="C38">
-        <v>-875.5336219114403</v>
+        <v>-827.0145529457544</v>
       </c>
       <c r="D38">
-        <v>-862.1240280423416</v>
+        <v>-819.9136699669799</v>
       </c>
       <c r="E38">
-        <v>-821.3995521598687</v>
+        <v>-721.4654396410991</v>
       </c>
       <c r="F38">
-        <v>-832.2955026027961</v>
+        <v>-731.0200347407787</v>
       </c>
       <c r="G38">
-        <v>-818.45993801782</v>
+        <v>-726.5750074680917</v>
       </c>
     </row>
     <row r="39">
@@ -1323,22 +1323,22 @@
         </is>
       </c>
       <c r="B39">
-        <v>-1114.19992565157</v>
+        <v>-1018.786350016695</v>
       </c>
       <c r="C39">
-        <v>-1114.68078345812</v>
+        <v>-1020.315713304785</v>
       </c>
       <c r="D39">
-        <v>-1084.517021515279</v>
+        <v>-984.115063462905</v>
       </c>
       <c r="E39">
-        <v>-992.1341759945966</v>
+        <v>-907.4049200559929</v>
       </c>
       <c r="F39">
-        <v>-1001.690953292492</v>
+        <v>-944.5484834198885</v>
       </c>
       <c r="G39">
-        <v>-977.9887965624968</v>
+        <v>-916.4218724566757</v>
       </c>
     </row>
     <row r="40">
@@ -1348,22 +1348,22 @@
         </is>
       </c>
       <c r="B40">
-        <v>-1108.448037718125</v>
+        <v>-1037.586915818834</v>
       </c>
       <c r="C40">
-        <v>-1111.346276801625</v>
+        <v>-1043.953846992046</v>
       </c>
       <c r="D40">
-        <v>-1086.948667711258</v>
+        <v>-1017.93369515943</v>
       </c>
       <c r="E40">
-        <v>-1032.880417642588</v>
+        <v>-955.4667747953498</v>
       </c>
       <c r="F40">
-        <v>-1056.06839340971</v>
+        <v>-986.493725442191</v>
       </c>
       <c r="G40">
-        <v>-1031.184627373174</v>
+        <v>-965.1493371726231</v>
       </c>
     </row>
     <row r="41">
@@ -1373,22 +1373,22 @@
         </is>
       </c>
       <c r="B41">
-        <v>-1247.158450414131</v>
+        <v>-959.4235838848591</v>
       </c>
       <c r="C41">
-        <v>-1244.45142482599</v>
+        <v>-952.9433449420227</v>
       </c>
       <c r="D41">
-        <v>-1205.272824113013</v>
+        <v>-922.2382372596385</v>
       </c>
       <c r="E41">
-        <v>-1211.816499995431</v>
+        <v>-928.0240330178325</v>
       </c>
       <c r="F41">
-        <v>-1207.042244801424</v>
+        <v>-915.9342813196292</v>
       </c>
       <c r="G41">
-        <v>-1171.638398830264</v>
+        <v>-887.491263557169</v>
       </c>
     </row>
     <row r="42">
@@ -1398,22 +1398,22 @@
         </is>
       </c>
       <c r="B42">
-        <v>-1042.657933003492</v>
+        <v>-747.0794098525414</v>
       </c>
       <c r="C42">
-        <v>-1039.344550157249</v>
+        <v>-743.0517040370307</v>
       </c>
       <c r="D42">
-        <v>-1045.349577456398</v>
+        <v>-763.7362227373563</v>
       </c>
       <c r="E42">
-        <v>-726.5399065326659</v>
+        <v>-539.1866727545538</v>
       </c>
       <c r="F42">
-        <v>-725.7727016864421</v>
+        <v>-738.5319829517287</v>
       </c>
       <c r="G42">
-        <v>-732.7743105222114</v>
+        <v>-756.4729079154956</v>
       </c>
     </row>
     <row r="43">
@@ -1423,22 +1423,22 @@
         </is>
       </c>
       <c r="B43">
-        <v>-988.2385499045089</v>
+        <v>-927.1196352218652</v>
       </c>
       <c r="C43">
-        <v>-987.7328297476799</v>
+        <v>-928.2076082433542</v>
       </c>
       <c r="D43">
-        <v>-964.0828427935314</v>
+        <v>-912.8627131813415</v>
       </c>
       <c r="E43">
-        <v>-940.4621035288695</v>
+        <v>-867.7043940982566</v>
       </c>
       <c r="F43">
-        <v>-947.2662729110182</v>
+        <v>-865.3226134761486</v>
       </c>
       <c r="G43">
-        <v>-924.2374137050731</v>
+        <v>-853.9409500509502</v>
       </c>
     </row>
     <row r="44">
@@ -1448,22 +1448,22 @@
         </is>
       </c>
       <c r="B44">
-        <v>-1163.635387599475</v>
+        <v>-1059.749602665282</v>
       </c>
       <c r="C44">
-        <v>-1162.236678569436</v>
+        <v>-1055.740675715124</v>
       </c>
       <c r="D44">
-        <v>-1134.214077596878</v>
+        <v>-1021.889945617577</v>
       </c>
       <c r="E44">
-        <v>-1119.535154017464</v>
+        <v>-1033.630801373522</v>
       </c>
       <c r="F44">
-        <v>-1124.68213044025</v>
+        <v>-1021.092751758971</v>
       </c>
       <c r="G44">
-        <v>-1097.31218083099</v>
+        <v>-988.8141761699653</v>
       </c>
     </row>
     <row r="45">
@@ -1473,22 +1473,22 @@
         </is>
       </c>
       <c r="B45">
-        <v>-1131.850620978258</v>
+        <v>-827.8192189402881</v>
       </c>
       <c r="C45">
-        <v>-1130.861611718199</v>
+        <v>-821.959012845056</v>
       </c>
       <c r="D45">
-        <v>-1112.294505797327</v>
+        <v>-810.0819538361378</v>
       </c>
       <c r="E45">
-        <v>-1000.476408435872</v>
+        <v>-728.1650417745603</v>
       </c>
       <c r="F45">
-        <v>-1008.725074870312</v>
+        <v>-728.8735466010712</v>
       </c>
       <c r="G45">
-        <v>-993.1471114552585</v>
+        <v>-724.1812696790353</v>
       </c>
     </row>
     <row r="46">
@@ -1498,22 +1498,22 @@
         </is>
       </c>
       <c r="B46">
-        <v>-895.8434384203546</v>
+        <v>-998.1007466352263</v>
       </c>
       <c r="C46">
-        <v>-893.5153548967778</v>
+        <v>-991.4959016236361</v>
       </c>
       <c r="D46">
-        <v>-864.7040128843785</v>
+        <v>-952.757718494716</v>
       </c>
       <c r="E46">
-        <v>-893.1532684358757</v>
+        <v>-994.6704353796948</v>
       </c>
       <c r="F46">
-        <v>-892.0758586990034</v>
+        <v>-975.2556041541584</v>
       </c>
       <c r="G46">
-        <v>-867.0805853520254</v>
+        <v>-940.0537269515112</v>
       </c>
     </row>
     <row r="47">
@@ -1523,22 +1523,22 @@
         </is>
       </c>
       <c r="B47">
-        <v>-936.7608625020126</v>
+        <v>-762.9935701229347</v>
       </c>
       <c r="C47">
-        <v>-936.6751034221406</v>
+        <v>-763.1441235878272</v>
       </c>
       <c r="D47">
-        <v>-918.283144230337</v>
+        <v>-757.3079934873323</v>
       </c>
       <c r="E47">
-        <v>-808.819051228816</v>
+        <v>-627.2136629591095</v>
       </c>
       <c r="F47">
-        <v>-806.8418093972961</v>
+        <v>-619.8684741149833</v>
       </c>
       <c r="G47">
-        <v>-798.9373062845492</v>
+        <v>-631.1566020898845</v>
       </c>
     </row>
     <row r="48">
@@ -1548,22 +1548,22 @@
         </is>
       </c>
       <c r="B48">
-        <v>-865.1566477585776</v>
+        <v>-736.7493846583363</v>
       </c>
       <c r="C48">
-        <v>-864.939429485608</v>
+        <v>-735.9353161471466</v>
       </c>
       <c r="D48">
-        <v>-847.7806085460392</v>
+        <v>-732.1867292756019</v>
       </c>
       <c r="E48">
-        <v>-796.9184634819425</v>
+        <v>-694.1717381365269</v>
       </c>
       <c r="F48">
-        <v>-796.7285865933191</v>
+        <v>-692.9976420669451</v>
       </c>
       <c r="G48">
-        <v>-788.610572467149</v>
+        <v>-695.8791066759422</v>
       </c>
     </row>
     <row r="49">
@@ -1573,22 +1573,22 @@
         </is>
       </c>
       <c r="B49">
-        <v>-1110.117710034905</v>
+        <v>-1076.637246927155</v>
       </c>
       <c r="C49">
-        <v>-1108.870010922036</v>
+        <v>-1072.778504786047</v>
       </c>
       <c r="D49">
-        <v>-1079.03080879343</v>
+        <v>-1031.000996477701</v>
       </c>
       <c r="E49">
-        <v>-999.5015384758639</v>
+        <v>-997.7619918733802</v>
       </c>
       <c r="F49">
-        <v>-999.4519742140851</v>
+        <v>-989.3732113497656</v>
       </c>
       <c r="G49">
-        <v>-973.634550702021</v>
+        <v>-953.1834727177312</v>
       </c>
     </row>
     <row r="50">
@@ -1598,22 +1598,22 @@
         </is>
       </c>
       <c r="B50">
-        <v>-785.2239246884277</v>
+        <v>-726.0313804709875</v>
       </c>
       <c r="C50">
-        <v>-773.8859992774663</v>
+        <v>-796.6936447390997</v>
       </c>
       <c r="D50">
-        <v>-761.880780956851</v>
+        <v>-785.5172425826744</v>
       </c>
       <c r="E50">
-        <v>-763.9683607435853</v>
+        <v>-643.8148872190853</v>
       </c>
       <c r="F50">
-        <v>-766.3363253765909</v>
+        <v>-647.1836285387053</v>
       </c>
       <c r="G50">
-        <v>-760.7663208504368</v>
+        <v>-649.1970460972193</v>
       </c>
     </row>
     <row r="51">
@@ -1623,22 +1623,22 @@
         </is>
       </c>
       <c r="B51">
-        <v>-1079.270211853246</v>
+        <v>-866.6245473504024</v>
       </c>
       <c r="C51">
-        <v>-1076.437067846696</v>
+        <v>-858.4724227492541</v>
       </c>
       <c r="D51">
-        <v>-1044.184016351575</v>
+        <v>-824.7106866507676</v>
       </c>
       <c r="E51">
-        <v>-990.2205753699637</v>
+        <v>-809.9377254427772</v>
       </c>
       <c r="F51">
-        <v>-991.7733675432888</v>
+        <v>-789.2136899188015</v>
       </c>
       <c r="G51">
-        <v>-969.0744471895583</v>
+        <v>-763.1398179795594</v>
       </c>
     </row>
   </sheetData>

</xml_diff>